<commit_message>
General updates and BF duration data
</commit_message>
<xml_diff>
--- a/data/country_baselines/Updated/Baseline information_Zambia SS.xlsx
+++ b/data/country_baselines/Updated/Baseline information_Zambia SS.xlsx
@@ -417,10 +417,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>